<commit_message>
docs: add question 2
</commit_message>
<xml_diff>
--- a/docs/excel/Definición del contrato de la API.xlsx
+++ b/docs/excel/Definición del contrato de la API.xlsx
@@ -1,12 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\oscar.lasso-m\Downloads\DOSW_ParcialT2_JoseMartinez\docs\excel\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{118CB781-43CA-4626-8D26-0812788B690C}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Hoja 1" sheetId="1" r:id="rId5"/>
+    <sheet name="Hoja 1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
@@ -228,32 +237,32 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="5">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <sz val="11.0"/>
+      <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
     </font>
     <font>
-      <sz val="11.0"/>
+      <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF1A1A1A"/>
       <name val="Arial"/>
     </font>
@@ -263,7 +272,7 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -273,7 +282,13 @@
     </fill>
   </fills>
   <borders count="2">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
     <border>
       <left style="thin">
         <color rgb="FFD9D9D9"/>
@@ -287,40 +302,44 @@
       <bottom style="thin">
         <color rgb="FFD9D9D9"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="6">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="1" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
@@ -328,7 +347,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -518,29 +537,32 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:S41"/>
+  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col customWidth="1" min="2" max="2" width="18.13"/>
-    <col customWidth="1" min="3" max="3" width="28.63"/>
-    <col customWidth="1" min="4" max="4" width="20.13"/>
-    <col customWidth="1" min="5" max="5" width="16.25"/>
-    <col customWidth="1" min="6" max="6" width="41.63"/>
-    <col customWidth="1" min="7" max="7" width="29.63"/>
-    <col customWidth="1" min="8" max="8" width="24.0"/>
-    <col customWidth="1" min="9" max="9" width="27.0"/>
-    <col customWidth="1" min="10" max="10" width="25.0"/>
-    <col customWidth="1" min="11" max="11" width="39.38"/>
+    <col min="2" max="2" width="18.140625" customWidth="1"/>
+    <col min="3" max="3" width="28.5703125" customWidth="1"/>
+    <col min="4" max="4" width="20.140625" customWidth="1"/>
+    <col min="5" max="5" width="16.28515625" customWidth="1"/>
+    <col min="6" max="6" width="41.5703125" customWidth="1"/>
+    <col min="7" max="7" width="29.5703125" customWidth="1"/>
+    <col min="8" max="8" width="30" customWidth="1"/>
+    <col min="9" max="9" width="27" customWidth="1"/>
+    <col min="10" max="10" width="25" customWidth="1"/>
+    <col min="11" max="11" width="39.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:19" ht="30" x14ac:dyDescent="0.2">
       <c r="A1" s="1"/>
       <c r="B1" s="2" t="s">
         <v>0</v>
@@ -573,7 +595,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:19" ht="105" x14ac:dyDescent="0.2">
       <c r="A2" s="1"/>
       <c r="B2" s="3" t="s">
         <v>10</v>
@@ -606,7 +628,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:19" ht="180" x14ac:dyDescent="0.2">
       <c r="A3" s="1"/>
       <c r="B3" s="3" t="s">
         <v>20</v>
@@ -639,7 +661,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:19" ht="105" x14ac:dyDescent="0.2">
       <c r="A4" s="1"/>
       <c r="B4" s="3" t="s">
         <v>29</v>
@@ -672,7 +694,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:19" ht="105" x14ac:dyDescent="0.2">
       <c r="A5" s="1"/>
       <c r="B5" s="3" t="s">
         <v>38</v>
@@ -705,7 +727,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:19" ht="90" x14ac:dyDescent="0.2">
       <c r="A6" s="1"/>
       <c r="B6" s="3" t="s">
         <v>44</v>
@@ -738,7 +760,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A7" s="1"/>
       <c r="B7" s="4"/>
       <c r="C7" s="5"/>
@@ -751,7 +773,7 @@
       <c r="J7" s="1"/>
       <c r="K7" s="1"/>
     </row>
-    <row r="8">
+    <row r="8" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A8" s="1"/>
       <c r="B8" s="4"/>
       <c r="C8" s="5"/>
@@ -764,7 +786,7 @@
       <c r="J8" s="1"/>
       <c r="K8" s="1"/>
     </row>
-    <row r="9">
+    <row r="9" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A9" s="1"/>
       <c r="B9" s="4"/>
       <c r="C9" s="5"/>
@@ -777,7 +799,7 @@
       <c r="J9" s="1"/>
       <c r="K9" s="1"/>
     </row>
-    <row r="10">
+    <row r="10" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A10" s="1"/>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
@@ -791,7 +813,7 @@
       <c r="K10" s="1"/>
       <c r="L10" s="1"/>
     </row>
-    <row r="11">
+    <row r="11" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A11" s="1"/>
       <c r="B11" s="4"/>
       <c r="C11" s="5"/>
@@ -804,7 +826,7 @@
       <c r="J11" s="1"/>
       <c r="K11" s="1"/>
     </row>
-    <row r="12">
+    <row r="12" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A12" s="1"/>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
@@ -825,7 +847,7 @@
       <c r="R12" s="1"/>
       <c r="S12" s="1"/>
     </row>
-    <row r="13">
+    <row r="13" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A13" s="1"/>
       <c r="B13" s="5"/>
       <c r="C13" s="5"/>
@@ -846,7 +868,7 @@
       <c r="R13" s="1"/>
       <c r="S13" s="1"/>
     </row>
-    <row r="14">
+    <row r="14" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A14" s="1"/>
       <c r="B14" s="5"/>
       <c r="C14" s="5"/>
@@ -867,7 +889,7 @@
       <c r="R14" s="1"/>
       <c r="S14" s="1"/>
     </row>
-    <row r="15">
+    <row r="15" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A15" s="1"/>
       <c r="B15" s="5"/>
       <c r="C15" s="5"/>
@@ -888,7 +910,7 @@
       <c r="R15" s="1"/>
       <c r="S15" s="1"/>
     </row>
-    <row r="16">
+    <row r="16" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A16" s="1"/>
       <c r="B16" s="5"/>
       <c r="C16" s="5"/>
@@ -909,7 +931,7 @@
       <c r="R16" s="1"/>
       <c r="S16" s="1"/>
     </row>
-    <row r="17">
+    <row r="17" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A17" s="1"/>
       <c r="B17" s="5"/>
       <c r="C17" s="5"/>
@@ -930,7 +952,7 @@
       <c r="R17" s="1"/>
       <c r="S17" s="1"/>
     </row>
-    <row r="18">
+    <row r="18" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A18" s="1"/>
       <c r="B18" s="5"/>
       <c r="C18" s="5"/>
@@ -951,7 +973,7 @@
       <c r="R18" s="1"/>
       <c r="S18" s="1"/>
     </row>
-    <row r="19">
+    <row r="19" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A19" s="1"/>
       <c r="B19" s="5"/>
       <c r="C19" s="5"/>
@@ -972,7 +994,7 @@
       <c r="R19" s="1"/>
       <c r="S19" s="1"/>
     </row>
-    <row r="20">
+    <row r="20" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A20" s="1"/>
       <c r="B20" s="5"/>
       <c r="C20" s="5"/>
@@ -993,7 +1015,7 @@
       <c r="R20" s="1"/>
       <c r="S20" s="1"/>
     </row>
-    <row r="21">
+    <row r="21" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A21" s="1"/>
       <c r="B21" s="5"/>
       <c r="C21" s="5"/>
@@ -1014,7 +1036,7 @@
       <c r="R21" s="1"/>
       <c r="S21" s="1"/>
     </row>
-    <row r="22">
+    <row r="22" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A22" s="1"/>
       <c r="B22" s="5"/>
       <c r="C22" s="5"/>
@@ -1035,7 +1057,7 @@
       <c r="R22" s="1"/>
       <c r="S22" s="1"/>
     </row>
-    <row r="23">
+    <row r="23" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A23" s="1"/>
       <c r="B23" s="5"/>
       <c r="C23" s="5"/>
@@ -1056,7 +1078,7 @@
       <c r="R23" s="1"/>
       <c r="S23" s="1"/>
     </row>
-    <row r="24">
+    <row r="24" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A24" s="1"/>
       <c r="B24" s="5"/>
       <c r="C24" s="5"/>
@@ -1077,7 +1099,7 @@
       <c r="R24" s="1"/>
       <c r="S24" s="1"/>
     </row>
-    <row r="25">
+    <row r="25" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A25" s="1"/>
       <c r="B25" s="5"/>
       <c r="C25" s="5"/>
@@ -1098,7 +1120,7 @@
       <c r="R25" s="1"/>
       <c r="S25" s="1"/>
     </row>
-    <row r="26">
+    <row r="26" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A26" s="1"/>
       <c r="B26" s="5"/>
       <c r="C26" s="5"/>
@@ -1119,7 +1141,7 @@
       <c r="R26" s="1"/>
       <c r="S26" s="1"/>
     </row>
-    <row r="27">
+    <row r="27" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A27" s="1"/>
       <c r="B27" s="5"/>
       <c r="C27" s="5"/>
@@ -1140,7 +1162,7 @@
       <c r="R27" s="1"/>
       <c r="S27" s="1"/>
     </row>
-    <row r="28">
+    <row r="28" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A28" s="1"/>
       <c r="B28" s="5"/>
       <c r="C28" s="5"/>
@@ -1161,7 +1183,7 @@
       <c r="R28" s="1"/>
       <c r="S28" s="1"/>
     </row>
-    <row r="29">
+    <row r="29" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A29" s="1"/>
       <c r="B29" s="5"/>
       <c r="C29" s="5"/>
@@ -1182,7 +1204,7 @@
       <c r="R29" s="1"/>
       <c r="S29" s="1"/>
     </row>
-    <row r="30">
+    <row r="30" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A30" s="1"/>
       <c r="B30" s="5"/>
       <c r="C30" s="5"/>
@@ -1203,7 +1225,7 @@
       <c r="R30" s="1"/>
       <c r="S30" s="1"/>
     </row>
-    <row r="31">
+    <row r="31" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A31" s="1"/>
       <c r="B31" s="5"/>
       <c r="C31" s="5"/>
@@ -1224,7 +1246,7 @@
       <c r="R31" s="1"/>
       <c r="S31" s="1"/>
     </row>
-    <row r="32">
+    <row r="32" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A32" s="1"/>
       <c r="B32" s="5"/>
       <c r="C32" s="5"/>
@@ -1245,7 +1267,7 @@
       <c r="R32" s="1"/>
       <c r="S32" s="1"/>
     </row>
-    <row r="33">
+    <row r="33" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A33" s="1"/>
       <c r="B33" s="5"/>
       <c r="C33" s="5"/>
@@ -1266,7 +1288,7 @@
       <c r="R33" s="1"/>
       <c r="S33" s="1"/>
     </row>
-    <row r="34">
+    <row r="34" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A34" s="1"/>
       <c r="B34" s="5"/>
       <c r="C34" s="5"/>
@@ -1287,7 +1309,7 @@
       <c r="R34" s="1"/>
       <c r="S34" s="1"/>
     </row>
-    <row r="35">
+    <row r="35" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A35" s="1"/>
       <c r="B35" s="5"/>
       <c r="C35" s="1"/>
@@ -1300,7 +1322,7 @@
       <c r="J35" s="1"/>
       <c r="K35" s="1"/>
     </row>
-    <row r="36">
+    <row r="36" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A36" s="1"/>
       <c r="B36" s="1"/>
       <c r="C36" s="1"/>
@@ -1313,7 +1335,7 @@
       <c r="J36" s="1"/>
       <c r="K36" s="1"/>
     </row>
-    <row r="37">
+    <row r="37" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A37" s="1"/>
       <c r="B37" s="1"/>
       <c r="C37" s="1"/>
@@ -1326,7 +1348,7 @@
       <c r="J37" s="1"/>
       <c r="K37" s="1"/>
     </row>
-    <row r="38">
+    <row r="38" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A38" s="1"/>
       <c r="B38" s="1"/>
       <c r="C38" s="1"/>
@@ -1339,7 +1361,7 @@
       <c r="J38" s="1"/>
       <c r="K38" s="1"/>
     </row>
-    <row r="39">
+    <row r="39" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A39" s="1"/>
       <c r="B39" s="1"/>
       <c r="C39" s="1"/>
@@ -1352,7 +1374,7 @@
       <c r="J39" s="1"/>
       <c r="K39" s="1"/>
     </row>
-    <row r="40">
+    <row r="40" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A40" s="1"/>
       <c r="B40" s="1"/>
       <c r="C40" s="1"/>
@@ -1365,10 +1387,10 @@
       <c r="J40" s="1"/>
       <c r="K40" s="1"/>
     </row>
-    <row r="41">
+    <row r="41" spans="1:19" x14ac:dyDescent="0.2">
       <c r="B41" s="1"/>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>